<commit_message>
feat: sync placement excel templates, add hackathon type, update 20min gatepass, and show completed drive status
</commit_message>
<xml_diff>
--- a/public/upload/round result.xlsx
+++ b/public/upload/round result.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30026"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="20417"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/bbf9f9cc0244fb7d/Documents/SCOPE Data/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User\Downloads\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="4" documentId="8_{D8322B61-2C58-44A8-B15F-D32A21D1E1F5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{103EA0CA-8E1A-43C3-B5A1-21917AF3A4DE}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A13F4440-F504-4B04-BFBE-16B5943DE584}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2304" yWindow="2304" windowWidth="17280" windowHeight="8880" xr2:uid="{8C4BDE77-E92D-42A4-A7C6-D7F972370E9A}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="23040" windowHeight="8772" xr2:uid="{8C4BDE77-E92D-42A4-A7C6-D7F972370E9A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,57 +20,106 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
-    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
-      <xcalcf:calcFeatures>
-        <xcalcf:feature name="microsoft.com:RD"/>
-        <xcalcf:feature name="microsoft.com:Single"/>
-        <xcalcf:feature name="microsoft.com:FV"/>
-        <xcalcf:feature name="microsoft.com:CNMTM"/>
-        <xcalcf:feature name="microsoft.com:LET_WF"/>
-      </xcalcf:calcFeatures>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
-  <si>
-    <t>Enrollment Number</t>
-  </si>
-  <si>
-    <t>Name</t>
-  </si>
-  <si>
-    <t>Email</t>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="16">
+  <si>
+    <t>Ghanshyam Dhote</t>
+  </si>
+  <si>
+    <t>Shubham Patel</t>
+  </si>
+  <si>
+    <t>Shivam Davande</t>
+  </si>
+  <si>
+    <t>0187CS231084</t>
+  </si>
+  <si>
+    <t>0187CS231220</t>
+  </si>
+  <si>
+    <t>0187CS231214</t>
   </si>
   <si>
     <t>2023-27</t>
   </si>
   <si>
-    <t>Batch</t>
-  </si>
-  <si>
-    <t>Department</t>
-  </si>
-  <si>
-    <t>Ghanshyam Dhote</t>
-  </si>
-  <si>
-    <t>0187CS231084</t>
-  </si>
-  <si>
-    <t>dhoteghanshyam9@gmail.com</t>
-  </si>
-  <si>
     <t>Computer-Science</t>
+  </si>
+  <si>
+    <t>AIDS</t>
+  </si>
+  <si>
+    <t>Cyber</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Cambria"/>
+        <family val="1"/>
+      </rPr>
+      <t>Sr. No</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Cambria"/>
+        <family val="1"/>
+      </rPr>
+      <t>Roll No</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Cambria"/>
+        <family val="1"/>
+      </rPr>
+      <t>Full Name</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Cambria"/>
+        <family val="1"/>
+      </rPr>
+      <t>Branch</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <rFont val="Cambria"/>
+        <family val="1"/>
+      </rPr>
+      <t>Campus</t>
+    </r>
+  </si>
+  <si>
+    <t>SISTec</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -91,21 +140,52 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="Cambria"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="12"/>
+      <name val="Cambria"/>
+      <family val="1"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill patternType="none"/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFBFBFBF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
       <top/>
       <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="FF000000"/>
+      </left>
+      <right style="thin">
+        <color rgb="FF000000"/>
+      </right>
+      <top style="thin">
+        <color rgb="FF000000"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FF000000"/>
+      </bottom>
       <diagonal/>
     </border>
   </borders>
@@ -116,12 +196,15 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="2"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="3">
     <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
@@ -438,7 +521,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F38EC05D-74E3-4953-81FD-B9F4B9431550}">
-  <dimension ref="A1:F2"/>
+  <dimension ref="A1:F9"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="16.6640625" customWidth="1"/>
@@ -447,45 +530,87 @@
     <col min="5" max="5" width="18.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A1" s="1" t="s">
+    <row r="1" spans="1:6" ht="15" x14ac:dyDescent="0.3">
+      <c r="A1" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B1" s="3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C1" s="3" t="s">
+        <v>12</v>
+      </c>
+      <c r="D1" s="3" t="s">
+        <v>13</v>
+      </c>
+      <c r="E1" s="3" t="s">
+        <v>14</v>
+      </c>
+      <c r="F1" s="1"/>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B2" t="s">
+        <v>3</v>
+      </c>
+      <c r="C2" t="s">
+        <v>0</v>
+      </c>
+      <c r="D2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="E2" t="s">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B3" t="s">
+        <v>4</v>
+      </c>
+      <c r="C3" t="s">
         <v>1</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="D3" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="E3" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="B4" t="s">
+        <v>5</v>
+      </c>
+      <c r="C4" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
-        <v>5</v>
-      </c>
-      <c r="E1" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="F1" s="1"/>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A2" t="s">
+      <c r="D4" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="E4" t="s">
         <v>6</v>
       </c>
-      <c r="B2" t="s">
-        <v>7</v>
-      </c>
-      <c r="C2" s="2" t="s">
-        <v>8</v>
-      </c>
-      <c r="D2" s="2" t="s">
-        <v>9</v>
-      </c>
-      <c r="E2" t="s">
-        <v>3</v>
-      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C7" s="2"/>
+      <c r="D7" s="2"/>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C8" s="2"/>
+      <c r="D8" s="2"/>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
     </row>
   </sheetData>
-  <hyperlinks>
-    <hyperlink ref="C2" r:id="rId1" xr:uid="{AFEB6CBE-5F23-4E66-ABC6-C61E9C8007FF}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>